<commit_message>
Complete AI suburb snapshot launch pack
</commit_message>
<xml_diff>
--- a/content/member-assets/realtor-suburb-snapshot/suburb-snapshot-pricing-calculator.xlsx
+++ b/content/member-assets/realtor-suburb-snapshot/suburb-snapshot-pricing-calculator.xlsx
@@ -185,7 +185,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>What this is</t>
@@ -257,7 +257,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" t="inlineStr" s="6">
         <is>
           <t>How to use</t>
@@ -269,7 +269,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
           <t>Delivery standards</t>
@@ -314,7 +314,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="54" customHeight="1">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -324,7 +324,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -334,7 +334,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -344,7 +344,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -806,7 +806,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Price forecasts</t>
@@ -875,9 +875,9 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -915,30 +915,30 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t>Source research hours</t>
+          <t>AI research + verification hours</t>
         </is>
       </c>
       <c r="B3" s="4">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="C3" t="inlineStr" s="2">
         <is>
-          <t>Public data collection and source log</t>
+          <t>One-prompt research, citation checks, and source ledger</t>
         </is>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
-          <t>Writing hours</t>
+          <t>Production hours</t>
         </is>
       </c>
       <c r="B4" s="8">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="C4" t="inlineStr" s="6">
         <is>
-          <t>Snapshot, talking points, email intro, captions</t>
+          <t>Template, talking points, email, captions, and export</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" t="inlineStr" s="6">
         <is>
           <t>Scope</t>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>Boundary</t>
@@ -1075,7 +1075,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Approval</t>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>Not included</t>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>Prospect context</t>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>Priority decision</t>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>Approval point</t>
@@ -1206,7 +1206,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
           <t>Upsell path</t>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3" ht="54" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t>2. Draft</t>
@@ -1313,7 +1313,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4" ht="54" customHeight="1">
       <c r="A4" t="inlineStr" s="6">
         <is>
           <t>3. Flag</t>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t>4. Approve</t>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="54" customHeight="1">
       <c r="A6" t="inlineStr" s="6">
         <is>
           <t>5. Deliver</t>

</xml_diff>